<commit_message>
:poop: Rework with ChatGPT 2
</commit_message>
<xml_diff>
--- a/assets/OutputData.xlsx
+++ b/assets/OutputData.xlsx
@@ -410,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -458,55 +458,9 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>79049004</v>
-      </c>
-      <c r="B3" s="1">
-        <v>45639.31736111111</v>
-      </c>
-      <c r="C3" s="1">
-        <v>45640.4375</v>
-      </c>
-      <c r="D3" s="2">
-        <v>-0.6</v>
-      </c>
-      <c r="E3" s="2">
-        <v>2.8</v>
-      </c>
-      <c r="F3" s="2">
-        <v>1.72</v>
-      </c>
-      <c r="G3" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>79049004</v>
-      </c>
-      <c r="B4" s="1">
-        <v>45640.4375</v>
-      </c>
-      <c r="C4" s="1">
-        <v>45641.34861111111</v>
-      </c>
-      <c r="D4" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="E4" s="2">
-        <v>7.1</v>
-      </c>
-      <c r="F4" s="2">
-        <v>4.51</v>
-      </c>
-      <c r="G4" s="2">
-        <v>4.6</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
weatherScraper : Move and add TU ans saved files
</commit_message>
<xml_diff>
--- a/assets/OutputData.xlsx
+++ b/assets/OutputData.xlsx
@@ -410,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -440,27 +440,50 @@
         <v>79049004</v>
       </c>
       <c r="B2" s="1">
-        <v>45638.32013888889</v>
+        <v>45669.35486111111</v>
       </c>
       <c r="C2" s="1">
-        <v>45639.31736111111</v>
+        <v>45670.31597222222</v>
       </c>
       <c r="D2" s="2">
-        <v>-0.7</v>
+        <v>-2.8</v>
       </c>
       <c r="E2" s="2">
-        <v>5.5</v>
+        <v>3</v>
       </c>
       <c r="F2" s="2">
-        <v>1.8</v>
+        <v>0.17</v>
       </c>
       <c r="G2" s="2">
-        <v>1.3</v>
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>79049004</v>
+      </c>
+      <c r="B3" s="1">
+        <v>45670.31597222222</v>
+      </c>
+      <c r="C3" s="1">
+        <v>45671.336805555555</v>
+      </c>
+      <c r="D3" s="2">
+        <v>-5.4</v>
+      </c>
+      <c r="E3" s="2">
+        <v>3.5</v>
+      </c>
+      <c r="F3" s="2">
+        <v>-1.48</v>
+      </c>
+      <c r="G3" s="2">
+        <v>-2</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>